<commit_message>
publish: workflow_dispatch main (88621e8)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-v1.0.0-rc1-dev.xlsx
+++ b/draft/testing-criteria-scorecard-v1.0.0-rc1-dev.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version v1.0.0-rc1+dev · branch main · commit 88621e8 (built 2026-10-15 01:33 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version v1.0.0-rc1+dev · branch main · commit 88621e8 (built 2026-10-15 01:36 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2259,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:33 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -7375,7 +7375,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:33 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -12354,7 +12354,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:33 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -14485,7 +14485,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:33 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -27254,7 +27254,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:33 UTC&amp;C&amp;"Arial,Regular"&amp;7 HIE System Validation Testing Criteria — Printed Evaluation Report&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;C&amp;"Arial,Regular"&amp;7 HIE System Validation Testing Criteria — Printed Evaluation Report&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -28558,7 +28558,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:33 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -29148,7 +29148,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:33 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -32450,7 +32450,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:33 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -33630,7 +33630,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:33 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -35123,7 +35123,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:33 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -37289,7 +37289,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:33 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -42560,7 +42560,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:33 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -46768,7 +46768,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:33 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
publish: push main (073e132)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-v1.0.0-rc1-dev.xlsx
+++ b/draft/testing-criteria-scorecard-v1.0.0-rc1-dev.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version v1.0.0-rc1+dev · branch main · commit 88621e8 (built 2026-10-15 01:36 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version v1.0.0-rc1+dev · branch main · commit 073e132 (built 2026-10-15 03:13 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2259,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -7375,7 +7375,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -12354,7 +12354,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -14485,7 +14485,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -27254,7 +27254,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;C&amp;"Arial,Regular"&amp;7 HIE System Validation Testing Criteria — Printed Evaluation Report&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;C&amp;"Arial,Regular"&amp;7 HIE System Validation Testing Criteria — Printed Evaluation Report&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -28558,7 +28558,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -29148,7 +29148,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -32450,7 +32450,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -33630,7 +33630,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -35123,7 +35123,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -37289,7 +37289,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -42560,7 +42560,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -46768,7 +46768,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 88621e8 · built 2026-10-15 01:36 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
publish: workflow_dispatch main (073e132)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-v1.0.0-rc1-dev.xlsx
+++ b/draft/testing-criteria-scorecard-v1.0.0-rc1-dev.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version v1.0.0-rc1+dev · branch main · commit 073e132 (built 2026-10-15 03:13 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version v1.0.0-rc1+dev · branch main · commit 073e132 (built 2026-10-15 03:16 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2259,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:16 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -7375,7 +7375,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:16 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -12354,7 +12354,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:16 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -14485,7 +14485,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:16 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -27254,7 +27254,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;C&amp;"Arial,Regular"&amp;7 HIE System Validation Testing Criteria — Printed Evaluation Report&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:16 UTC&amp;C&amp;"Arial,Regular"&amp;7 HIE System Validation Testing Criteria — Printed Evaluation Report&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -28558,7 +28558,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:16 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -29148,7 +29148,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:16 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -32450,7 +32450,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:16 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -33630,7 +33630,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:16 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -35123,7 +35123,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:16 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -37289,7 +37289,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:16 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -42560,7 +42560,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:16 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -46768,7 +46768,7 @@
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:13 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddFooter>&amp;L&amp;8 Version v1.0.0-rc1+dev · branch main · commit 073e132 · built 2026-10-15 03:16 UTC&amp;R&amp;8 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
publish: push main (8686fca)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-v1.0.0-rc1-dev.xlsx
+++ b/draft/testing-criteria-scorecard-v1.0.0-rc1-dev.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version v1.0.0-rc1+dev · branch main · commit 0d164db (built 2026-10-15 03:19 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version v1.0.0-rc1+dev · branch main · commit 8686fca (built 2026-10-15 03:39 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 0d164db · built 2026-10-15 03:19 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7374,7 +7374,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 0d164db · built 2026-10-15 03:19 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12353,7 +12353,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 0d164db · built 2026-10-15 03:19 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14484,7 +14484,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 0d164db · built 2026-10-15 03:19 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27253,7 +27253,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 0d164db · built 2026-10-15 03:19 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28557,7 +28557,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 0d164db · built 2026-10-15 03:19 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29147,7 +29147,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 0d164db · built 2026-10-15 03:19 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32449,7 +32449,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 0d164db · built 2026-10-15 03:19 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33629,7 +33629,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 0d164db · built 2026-10-15 03:19 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35122,7 +35122,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 0d164db · built 2026-10-15 03:19 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37288,7 +37288,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 0d164db · built 2026-10-15 03:19 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42559,7 +42559,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 0d164db · built 2026-10-15 03:19 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46767,7 +46767,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 0d164db · built 2026-10-15 03:19 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push main (7c46fb5)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-v1.0.0-rc1-dev.xlsx
+++ b/draft/testing-criteria-scorecard-v1.0.0-rc1-dev.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version v1.0.0-rc1+dev · branch main · commit 8686fca (built 2026-10-15 03:39 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 (built 2026-10-15 03:56 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7374,7 +7374,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12353,7 +12353,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14484,7 +14484,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27253,7 +27253,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28557,7 +28557,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29147,7 +29147,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32449,7 +32449,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33629,7 +33629,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35122,7 +35122,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37288,7 +37288,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42559,7 +42559,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46767,7 +46767,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 8686fca · built 2026-10-15 03:39 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: workflow_dispatch main (7c46fb5)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-v1.0.0-rc1-dev.xlsx
+++ b/draft/testing-criteria-scorecard-v1.0.0-rc1-dev.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 (built 2026-10-15 03:56 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 (built 2026-10-15 04:26 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 04:26 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7374,7 +7374,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 04:26 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12353,7 +12353,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 04:26 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14484,7 +14484,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 04:26 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27253,7 +27253,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 04:26 UTC</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28557,7 +28557,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 04:26 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29147,7 +29147,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 04:26 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32449,7 +32449,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 04:26 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33629,7 +33629,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 04:26 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35122,7 +35122,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 04:26 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37288,7 +37288,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 04:26 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42559,7 +42559,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 04:26 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46767,7 +46767,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 03:56 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version v1.0.0-rc1+dev · branch main · commit 7c46fb5 · built 2026-10-15 04:26 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>